<commit_message>
updated the messy raw data
</commit_message>
<xml_diff>
--- a/inst/extdata/pe_2025_messy.xlsx
+++ b/inst/extdata/pe_2025_messy.xlsx
@@ -8,159 +8,153 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ernestcaballero/Developer/data501/peridial/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98EC08C4-F3F6-7041-BA6A-FC966C53C948}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80318411-7119-744C-BE34-27E07DA173F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PE" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="45">
   <si>
     <t>Patient ID</t>
   </si>
   <si>
-    <t>Date of Infection</t>
+    <t>Last Dose Antibiotic</t>
+  </si>
+  <si>
+    <t>Overnight Hospitalisation</t>
+  </si>
+  <si>
+    <t>Days Hospitalised</t>
+  </si>
+  <si>
+    <t>Interim HD</t>
+  </si>
+  <si>
+    <t>Permanent HD</t>
+  </si>
+  <si>
+    <t>First Dialysis Date</t>
+  </si>
+  <si>
+    <t>Last Dialysis Date</t>
+  </si>
+  <si>
+    <t>SPD0003</t>
+  </si>
+  <si>
+    <t>Staphylococcus  epidermidis</t>
+  </si>
+  <si>
+    <t>SPD0007</t>
+  </si>
+  <si>
+    <t>negative</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>SPD0012</t>
+  </si>
+  <si>
+    <t>e. coli</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  STAPHYLOCOCCUS AUREUS </t>
+  </si>
+  <si>
+    <t>SPD0018</t>
+  </si>
+  <si>
+    <t>Klebsiella sp.</t>
+  </si>
+  <si>
+    <t>SPD0023</t>
+  </si>
+  <si>
+    <t>S epidermidis</t>
+  </si>
+  <si>
+    <t>SPD0025</t>
+  </si>
+  <si>
+    <t>pseudomonas AERUGINOSA</t>
+  </si>
+  <si>
+    <t>SPD0030</t>
+  </si>
+  <si>
+    <t>Enterococcus faecalis</t>
+  </si>
+  <si>
+    <t>SPD0033</t>
+  </si>
+  <si>
+    <t>Culture negative</t>
+  </si>
+  <si>
+    <t>SPD0036</t>
+  </si>
+  <si>
+    <t>Coag - Neg Staph, Staph Epidermidis</t>
+  </si>
+  <si>
+    <t>SPD0041</t>
+  </si>
+  <si>
+    <t>Escherichia coli </t>
+  </si>
+  <si>
+    <t>SPD03</t>
+  </si>
+  <si>
+    <t>S. aureus</t>
+  </si>
+  <si>
+    <t>SPD0047</t>
+  </si>
+  <si>
+    <t>Streptococcus pneumoniae</t>
+  </si>
+  <si>
+    <t>SPD0052</t>
+  </si>
+  <si>
+    <t>K pneumoniae</t>
+  </si>
+  <si>
+    <t>SPD0055</t>
+  </si>
+  <si>
+    <t>staph epidermidis</t>
+  </si>
+  <si>
+    <t>SPD0056</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	Enterococcus faecium</t>
+  </si>
+  <si>
+    <t>SPD0058</t>
+  </si>
+  <si>
+    <t>S. epidermidis; Staph epidermidis</t>
+  </si>
+  <si>
+    <t>Culture Negative</t>
+  </si>
+  <si>
+    <t>Infection Date</t>
   </si>
   <si>
     <t>Organism</t>
-  </si>
-  <si>
-    <t>Last Dose Antibiotic</t>
-  </si>
-  <si>
-    <t>Overnight Hospitalisation</t>
-  </si>
-  <si>
-    <t>Days Hospitalised</t>
-  </si>
-  <si>
-    <t>Catheter Removed</t>
-  </si>
-  <si>
-    <t>Catheter Removed Date</t>
-  </si>
-  <si>
-    <t>Interim HD</t>
-  </si>
-  <si>
-    <t>Permanent HD</t>
-  </si>
-  <si>
-    <t>First Dialysis Date</t>
-  </si>
-  <si>
-    <t>Last Dialysis Date</t>
-  </si>
-  <si>
-    <t>SPD0003</t>
-  </si>
-  <si>
-    <t>Staphylococcus  epidermidis</t>
-  </si>
-  <si>
-    <t>SPD0007</t>
-  </si>
-  <si>
-    <t>negative</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>SPD0012</t>
-  </si>
-  <si>
-    <t>e. coli</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  STAPHYLOCOCCUS AUREUS </t>
-  </si>
-  <si>
-    <t>SPD0018</t>
-  </si>
-  <si>
-    <t>Klebsiella sp.</t>
-  </si>
-  <si>
-    <t>SPD0023</t>
-  </si>
-  <si>
-    <t>S epidermidis</t>
-  </si>
-  <si>
-    <t>SPD0025</t>
-  </si>
-  <si>
-    <t>pseudomonas AERUGINOSA</t>
-  </si>
-  <si>
-    <t>SPD0030</t>
-  </si>
-  <si>
-    <t>Enterococcus faecalis</t>
-  </si>
-  <si>
-    <t>SPD0033</t>
-  </si>
-  <si>
-    <t>Culture negative</t>
-  </si>
-  <si>
-    <t>SPD0036</t>
-  </si>
-  <si>
-    <t>Coag - Neg Staph, Staph Epidermidis</t>
-  </si>
-  <si>
-    <t>SPD0041</t>
-  </si>
-  <si>
-    <t>Escherichia coli </t>
-  </si>
-  <si>
-    <t>SPD03</t>
-  </si>
-  <si>
-    <t>S. aureus</t>
-  </si>
-  <si>
-    <t>SPD0047</t>
-  </si>
-  <si>
-    <t>Streptococcus pneumoniae</t>
-  </si>
-  <si>
-    <t>SPD0052</t>
-  </si>
-  <si>
-    <t>K pneumoniae</t>
-  </si>
-  <si>
-    <t>SPD0055</t>
-  </si>
-  <si>
-    <t>staph epidermidis</t>
-  </si>
-  <si>
-    <t>SPD0056</t>
-  </si>
-  <si>
-    <t xml:space="preserve">	Enterococcus faecium</t>
-  </si>
-  <si>
-    <t>SPD0058</t>
-  </si>
-  <si>
-    <t>S. epidermidis; Staph epidermidis</t>
-  </si>
-  <si>
-    <t>Culture Negative</t>
   </si>
 </sst>
 </file>
@@ -511,7 +505,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -520,328 +514,320 @@
     <col min="4" max="4" width="23" customWidth="1"/>
     <col min="5" max="5" width="28" customWidth="1"/>
     <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="19" customWidth="1"/>
-    <col min="8" max="8" width="24" customWidth="1"/>
-    <col min="9" max="9" width="13" customWidth="1"/>
-    <col min="10" max="10" width="15" customWidth="1"/>
-    <col min="11" max="11" width="22" customWidth="1"/>
-    <col min="12" max="12" width="21" customWidth="1"/>
+    <col min="7" max="7" width="13" customWidth="1"/>
+    <col min="8" max="8" width="15" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
+    <col min="10" max="10" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>12</v>
       </c>
       <c r="B2" s="2">
         <v>45698</v>
       </c>
       <c r="C2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D2" s="2">
         <v>45712</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B3" s="2">
         <v>45738</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D3" s="2">
         <v>45752</v>
       </c>
       <c r="E3" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F3">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B4" s="2">
         <v>45675</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D4" s="2">
         <v>45689</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B5" s="2">
         <v>45874</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D5" s="2">
         <v>45888</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B6" s="2">
         <v>45791</v>
       </c>
       <c r="C6" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D6" s="2">
         <v>45805</v>
       </c>
       <c r="E6" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F6">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B7" s="2">
         <v>45749</v>
       </c>
       <c r="C7" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D7" s="2">
         <v>45763</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B8" s="2">
         <v>45836</v>
       </c>
       <c r="C8" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D8" s="2">
         <v>45850</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B9" s="2">
         <v>45915</v>
       </c>
       <c r="C9" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B10" s="2">
         <v>45849</v>
       </c>
       <c r="C10" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B11" s="2">
         <v>45981</v>
       </c>
       <c r="C11" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D11" s="2">
         <v>45995</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B12" s="2">
         <v>45765</v>
       </c>
       <c r="C12" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D12" s="2">
         <v>45779</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B13" s="2">
         <v>45868</v>
       </c>
       <c r="C13" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D13" s="2">
         <v>45882</v>
       </c>
       <c r="E13" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F13">
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B14" s="2">
         <v>45935</v>
       </c>
       <c r="C14" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D14" s="2">
         <v>45949</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B15" s="2">
         <v>45759</v>
       </c>
       <c r="C15" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D15" s="2">
         <v>45773</v>
       </c>
       <c r="E15" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F15">
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B16" s="2">
         <v>45721</v>
       </c>
       <c r="C16" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D16" s="2">
         <v>45735</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B17" s="2">
         <v>45823</v>
       </c>
       <c r="C17" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="D17" s="2">
         <v>45837</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B18" s="2">
         <v>45797</v>
       </c>
       <c r="C18" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D18" s="2">
         <v>45811</v>
       </c>
-      <c r="I18" t="s">
-        <v>16</v>
-      </c>
-      <c r="K18" s="2">
+      <c r="G18" t="s">
+        <v>12</v>
+      </c>
+      <c r="I18" s="2">
         <v>45809</v>
       </c>
-      <c r="L18" s="2">
+      <c r="J18" s="2">
         <v>45823</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B19" s="2">
         <v>45976</v>
       </c>
       <c r="C19" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D19" s="2">
         <v>45990</v>

</xml_diff>